<commit_message>
feat: complete production workflows and navigation
</commit_message>
<xml_diff>
--- a/docs/examples/Accounting_Pack_Monthly_2026-08.xlsx
+++ b/docs/examples/Accounting_Pack_Monthly_2026-08.xlsx
@@ -7,11 +7,77 @@
     <sheet name="Worker direct costs" sheetId="3" r:id="rId3"/>
     <sheet name="Expenses" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Invoice register'!$A$1:$Q$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Invoice register'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Collections'!$A$1:$K$2</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Collections'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Worker direct costs'!$A$1:$O$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Worker direct costs'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Expenses'!$A$1:$R$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Expenses'!$1:$1</definedName>
+  </definedNames>
 </workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00;[Red]-#,##0.00"/>
+  </numFmts>
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+  </fonts>
+  <fills count="1">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border/>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="top"/>
+    </xf>
+  </cellXfs>
+</styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="11" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="25" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="15" customWidth="1"/>
+    <col min="11" max="11" width="10" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="10" customWidth="1"/>
+    <col min="15" max="15" width="10" customWidth="1" style="2"/>
+    <col min="16" max="16" width="10" customWidth="1" style="2"/>
+    <col min="17" max="17" width="10" customWidth="1" style="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -84,6 +150,21 @@
           <t>currency</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>net</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>gross</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -121,15 +202,11 @@
           <t>2026-08-01 → 2026-08-14</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
+      <c r="H2" s="1">
+        <v>46244</v>
+      </c>
+      <c r="I2" s="1">
+        <v>46275</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -155,6 +232,17 @@
         <is>
           <t>USD</t>
         </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>57437.25</v>
       </c>
     </row>
     <row r="3">
@@ -193,15 +281,11 @@
           <t>2026-08-01 → 2026-08-14</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
+      <c r="H3" s="1">
+        <v>46244</v>
+      </c>
+      <c r="I3" s="1">
+        <v>46275</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -228,13 +312,40 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>13363.31</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:Q3"/>
+  <printOptions horizontalCentered="0" verticalCentered="0"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1" style="2"/>
+    <col min="9" max="9" width="24" customWidth="1" style="2"/>
+    <col min="10" max="10" width="22" customWidth="1" style="2"/>
+    <col min="11" max="11" width="13" customWidth="1" style="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -272,6 +383,26 @@
           <t>reference</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>grossInvoiced</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>amountCollectedInMonth</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>totalCollectedToDate</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>outstanding</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -309,13 +440,53 @@
           <t>WF-REF-981245</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K2"/>
+  <printOptions horizontalCentered="0" verticalCentered="0"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="23" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="23" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="10" width="19" customWidth="1"/>
+    <col min="11" max="11" width="27" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1" style="2"/>
+    <col min="13" max="13" width="21" customWidth="1" style="2"/>
+    <col min="14" max="14" width="25" customWidth="1" style="2"/>
+    <col min="15" max="15" width="15" customWidth="1" style="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -373,6 +544,26 @@
           <t>approvedCompensationMinor</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>approvedCompensation</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>settledCompensation</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>internalLoadedLaborCost</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>reimbursement</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -405,16 +596,14 @@
           <t>131.50</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2">
+        <v>7890</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>7890</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>7890</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>USD</t>
@@ -428,6 +617,24 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>526000</t>
+        </is>
+      </c>
+      <c r="L2">
+        <v>5260</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -462,16 +669,14 @@
           <t>134.60</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3">
+        <v>8076</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>8076</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>8076</t>
-        </is>
-      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>USD</t>
@@ -485,6 +690,24 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>471100</t>
+        </is>
+      </c>
+      <c r="L3">
+        <v>4711</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -519,16 +742,14 @@
           <t>129.50</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4">
+        <v>7770</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>7770</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>7770</t>
-        </is>
-      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>USD</t>
@@ -542,6 +763,24 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>453250</t>
+        </is>
+      </c>
+      <c r="L4">
+        <v>4532.5</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -576,16 +815,14 @@
           <t>134.50</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5">
+        <v>8070</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>8070</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>8070</t>
-        </is>
-      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>USD</t>
@@ -599,6 +836,24 @@
       <c r="K5" t="inlineStr">
         <is>
           <t>470750</t>
+        </is>
+      </c>
+      <c r="L5">
+        <v>4707.5</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -633,16 +888,14 @@
           <t>130.60</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6">
+        <v>7836</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>7836</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>7836</t>
-        </is>
-      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>USD</t>
@@ -656,6 +909,24 @@
       <c r="K6" t="inlineStr">
         <is>
           <t>457100</t>
+        </is>
+      </c>
+      <c r="L6">
+        <v>4571</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -690,16 +961,14 @@
           <t>125.75</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7">
+        <v>7545</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>7545</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>7545</t>
-        </is>
-      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>USD</t>
@@ -713,6 +982,24 @@
       <c r="K7" t="inlineStr">
         <is>
           <t>440125</t>
+        </is>
+      </c>
+      <c r="L7">
+        <v>4401.25</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -747,16 +1034,14 @@
           <t>108.00</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8">
+        <v>6480</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>6480</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>6480</t>
-        </is>
-      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>USD</t>
@@ -770,6 +1055,24 @@
       <c r="K8" t="inlineStr">
         <is>
           <t>378000</t>
+        </is>
+      </c>
+      <c r="L8">
+        <v>3780</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -804,16 +1107,14 @@
           <t>114.00</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9">
+        <v>6840</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>6840</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>6840</t>
-        </is>
-      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>USD</t>
@@ -827,6 +1128,24 @@
       <c r="K9" t="inlineStr">
         <is>
           <t>399000</t>
+        </is>
+      </c>
+      <c r="L9">
+        <v>3990</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -861,16 +1180,14 @@
           <t>148.00</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10">
+        <v>8880</v>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>8880</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>8880</t>
-        </is>
-      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>USD</t>
@@ -886,13 +1203,54 @@
           <t>592000</t>
         </is>
       </c>
+      <c r="L10">
+        <v>5920</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:O10"/>
+  <printOptions horizontalCentered="0" verticalCentered="0"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="11" customWidth="1"/>
+    <col min="12" max="12" width="13" customWidth="1"/>
+    <col min="13" max="13" width="10" customWidth="1"/>
+    <col min="14" max="14" width="10" customWidth="1" style="2"/>
+    <col min="15" max="15" width="10" customWidth="1" style="2"/>
+    <col min="16" max="16" width="10" customWidth="1" style="2"/>
+    <col min="17" max="17" width="23" customWidth="1" style="2"/>
+    <col min="18" max="18" width="15" customWidth="1" style="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -960,18 +1318,41 @@
           <t>billable</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>gross</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>projectCurrencyAmount</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>billingAmount</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1">
+        <v>46236</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>American Airlines</t>
@@ -1027,18 +1408,37 @@
           <t>true</t>
         </is>
       </c>
+      <c r="N2">
+        <v>973.8</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P2">
+        <v>973.8</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>Hertz DFW</t>
@@ -1094,18 +1494,37 @@
           <t>true</t>
         </is>
       </c>
+      <c r="N3">
+        <v>258.98</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P3">
+        <v>258.98</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-08-04</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>Marriott Georgetown</t>
@@ -1161,18 +1580,37 @@
           <t>true</t>
         </is>
       </c>
+      <c r="N4">
+        <v>856.32</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P4">
+        <v>856.32</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1">
+        <v>46239</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>Chevron Fuel</t>
@@ -1228,7 +1666,31 @@
           <t>true</t>
         </is>
       </c>
+      <c r="N5">
+        <v>107.9</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P5">
+        <v>107.9</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:R5"/>
+  <printOptions horizontalCentered="0" verticalCentered="0"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
</xml_diff>